<commit_message>
fixed notes mode video loading
</commit_message>
<xml_diff>
--- a/database/Take Notes/RL/RL.xlsx
+++ b/database/Take Notes/RL/RL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cursor AI\database\Take Notes\RL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57E6282-4218-4CA2-9B8E-B7252A83C886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79FF580-3655-4ED8-8491-955CBDA46FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1631" uniqueCount="1095">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1632" uniqueCount="1096">
   <si>
     <t>ID</t>
   </si>
@@ -3926,6 +3926,9 @@
 Well done! Vehicle-dependent means needing vehicles to live and work.
 That's the end of the video!  
 I’m Bel — like and subscribe for Better English Learning!</t>
+  </si>
+  <si>
+    <t>https://youtu.be/1V0aZUO57xY</t>
   </si>
 </sst>
 </file>
@@ -4420,6 +4423,9 @@
       <c r="E5" s="3" t="s">
         <v>1094</v>
       </c>
+      <c r="F5" t="s">
+        <v>1095</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">

</xml_diff>

<commit_message>
Watch mode question UI fixed
</commit_message>
<xml_diff>
--- a/database/Take Notes/RL/RL.xlsx
+++ b/database/Take Notes/RL/RL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cursor AI\database\Take Notes\RL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79FF580-3655-4ED8-8491-955CBDA46FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C86EA3-987A-4656-943D-37BE15686436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1632" uniqueCount="1096">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1634" uniqueCount="1100">
   <si>
     <t>ID</t>
   </si>
@@ -3929,6 +3929,176 @@
   </si>
   <si>
     <t>https://youtu.be/1V0aZUO57xY</t>
+  </si>
+  <si>
+    <t>https://youtu.be/HoCzqTtCbJc</t>
+  </si>
+  <si>
+    <t>Host (Bel):
+Welcome to today’s learning podcast! I’m Bel, and I’m really happy you’re listening today.
+In this episode, we’re going to talk about what makes a city fair and just. This idea comes from philosophy, but don’t worry — we’re going to explain everything in a simple and clear way.
+When we talk about a “just city,” we are really asking some important questions.
+Who benefits from city policies?
+Who is helped the most?
+And who might be hurt?
+To help us explore these questions, I’m joined by Alison. Alison has studied philosophy and has spent a lot of time thinking about fairness, cities, and social policy.
+Alison, thank you so much for being here today.
+Expert (Alison):
+Thank you, Bel. I’m very happy to be here and to talk with your listeners.
+Host (Bel):
+So, Alison, let’s start at the beginning. For our listeners, can you explain how philosophy helped you think about what makes a city just?
+Expert (Alison):
+Of course. From reading philosophy, I came up with three guiding principles for a just city. These principles are equity, democracy, and diversity.
+Host (Bel):
+Three principles already give us a clear structure. For our listeners, where do these ideas come from?
+Expert (Alison):
+They come from the work of several philosophers. One philosopher who influenced me a lot is Ross.
+Host (Bel):
+Let me pause you there, because this is really important.
+You choose the word equity, not equality. Many of our listeners may think these words mean the same thing.
+Can you explain the difference to our listeners?
+Expert (Alison):
+Yes, this is a key idea.
+Equality means everyone gets the same thing.
+Equity means that policies should help people so that those who are worst off become better off.
+Host (Bel):
+So, just to make sure everyone is following — equity does not mean everyone must become equal?
+Expert (Alison):
+That’s right. Equity does not mean everyone is the same.
+But it does mean that no policy should make the most disadvantaged people even more disadvantaged.
+Host (Bel):
+That feels very powerful.
+So when we talk about city policies, when should we think about equity?
+Expert (Alison):
+We must think about equity at the moment the policy is created and used, not only in the future.
+Host (Bel):
+Can you explain that a bit more for our listeners?
+Expert (Alison):
+Sure. Sometimes people say, “We need to make our city more competitive now, and later the benefits will reach everyone.”
+But this does not justify hurting the weakest people today.
+Host (Bel):
+I think many listeners will recognize that idea.
+Expert (Alison):
+Yes. Around the world, we see examples where people’s homes are destroyed in the name of the “greater good.”
+They are told that one day they will benefit — but right now, they suffer.
+Host (Bel):
+So equity asks us to be very careful, doesn’t it?
+Expert (Alison):
+Exactly. Equity means we do not take advantage of people who are weakest, even if we say it is for a better future.
+Host (Bel):
+Let me say this again in simple words for our listeners.
+Equity means we should never improve a city by hurting the people who already have the least.
+Expert (Alison):
+Yes. That is exactly the heart of the idea.
+Host (Bel):
+Thank you so much, Alison, for explaining this so clearly.
+And thank you to our listeners for spending time with us today.
+If you want, next I can:
+✅ Add a listener recap + vocabulary section
+✅ Convert this into your standard Version 2 teaching script
+✅ Make it even more interactive (questions directly to the listener)
+✅ Simplify further to A2 only
+Just tell me what you’d like next 🎧✨</t>
+  </si>
+  <si>
+    <t>https://youtu.be/vY1V59_i82c</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Welcome to today’s learning podcast! I am Bel, and I’m really happy you’re listening today.
+In this episode, we’re talking about what makes a city fair and just. This idea comes from philosophy, but don’t worry, we’ll explain everything in a simple way.
+When we talk about a just city, we ask important questions. Who benefits from city policies? Who is helped the most? And who might be hurt?
+We're going to explore these ideas with Alison, a philosophy expert.
+So, how did philosophy help shape these ideas, Alison?
+From reading philosophy, three guiding principles for a just city were identified: equity, democracy, and diversity.
+These ideas come from the work of several philosophers. One important philosopher is Ross.
+You may be wondering: why use the word equity instead of equality?
+That’s a great question.
+Equality means everyone gets the same thing. Equity means helping people so that those who are worst off become better off.
+Equity does not mean everyone must be equal. But it does mean that no policy should make the most disadvantaged people more disadvantaged.
+So when should we think about equity?
+We need to think about equity at the time a policy is created, not only in the future.
+Sometimes people say, “We must make the city more competitive now, and later the benefits will reach everyone.”
+But this does not justify hurting the weakest people today.
+Around the world, we see examples of people losing their homes in the name of the greater good. They are told they will benefit one day, but they suffer now.
+Equity means we do not take advantage of people who are weakest.
+In simple words, equity means we should never improve a city by hurting the people who already have the least.
+Now let’s recap what we learned today.
+A just city is a fair city.
+Philosophy gives us three principles for a just city: equity, democracy, and diversity.
+Equity means helping the people who are worst off.
+Equity is different from equality.
+Good policies should not harm the weakest people, even in the name of the future.
+That's the main ideas that you learned today! We will now review some new vocabularies.
+Repeat after me.
+Just city
+&lt;break time="2s" /&gt;
+Just city
+&lt;break time="2s" /&gt;
+Just city
+&lt;break time="2s" /&gt;
+Good job! A just city is a city that is fair to everyone.
+&lt;break time="0.5s" /&gt;
+Next
+&lt;break time="0.5s" /&gt;
+Equity
+&lt;break time="2s" /&gt;
+Equity
+&lt;break time="2s" /&gt;
+Equity
+&lt;break time="2s" /&gt;
+Great! Equity means helping people so the weakest become better off.
+&lt;break time="0.5s" /&gt;
+Next
+&lt;break time="0.5s" /&gt;
+Equality
+&lt;break time="2s" /&gt;
+Equality
+&lt;break time="2s" /&gt;
+Equality
+&lt;break time="2s" /&gt;
+Well done! Equality means everyone gets the same thing.
+&lt;break time="0.5s" /&gt;
+Next
+&lt;break time="0.5s" /&gt;
+Policy
+&lt;break time="1s" /&gt;
+Policy
+&lt;break time="1s" /&gt;
+Policy
+&lt;break time="1s" /&gt;
+A policy is a plan or rule made by a government or city.
+&lt;break time="0.5s" /&gt;
+Next
+&lt;break time="0.5s" /&gt;
+Disadvantaged
+&lt;break time="1s" /&gt;
+Disadvantaged
+&lt;break time="1s" /&gt;
+Disadvantaged
+&lt;break time="1s" /&gt;
+Disadvantaged means having less help or fewer chances.
+&lt;break time="0.5s" /&gt;
+Next
+&lt;break time="0.5s" /&gt;
+Greater good
+&lt;break time="1s" /&gt;
+Greater good
+&lt;break time="1s" /&gt;
+Greater good
+&lt;break time="1s" /&gt;
+The greater good means helping many people, sometimes at a cost.
+&lt;break time="0.5s" /&gt;
+Next
+&lt;break time="0.5s" /&gt;
+Philosophy
+&lt;break time="1s" /&gt;
+Philosophy
+&lt;break time="1s" /&gt;
+Philosophy
+&lt;break time="1s" /&gt;
+Well done! Philosophy is the study of ideas about life, fairness, and meaning.
+That's the end of the video!
+I’m Bel — like and subscribe for Better English Learning!</t>
   </si>
 </sst>
 </file>
@@ -4015,8 +4185,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4403,8 +4573,8 @@
       <c r="E4" t="s">
         <v>1091</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>1088</v>
+      <c r="F4" s="3" t="s">
+        <v>1096</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -4417,10 +4587,10 @@
       <c r="C5" t="s">
         <v>545</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>1093</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" t="s">
         <v>1094</v>
       </c>
       <c r="F5" t="s">
@@ -4437,8 +4607,14 @@
       <c r="C6" t="s">
         <v>546</v>
       </c>
-      <c r="E6" t="s">
-        <v>1092</v>
+      <c r="D6" s="4" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1099</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>1098</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -11930,7 +12106,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F4" r:id="rId1" xr:uid="{FC924530-9D20-4B0C-8B08-C35D65377ECD}"/>
+    <hyperlink ref="F6" r:id="rId1" xr:uid="{E98772F5-F3A2-4178-B97F-E8A8C6014580}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
added SRS and Writing challenge
</commit_message>
<xml_diff>
--- a/database/Take Notes/RL/RL.xlsx
+++ b/database/Take Notes/RL/RL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cursor AI\database\Take Notes\RL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C590F8-9C35-4A49-8ACC-1E718FF65A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD172A36-C4F0-46D3-83EF-ABE0F90B7ADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1631" uniqueCount="1100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1632" uniqueCount="1101">
   <si>
     <t>ID</t>
   </si>
@@ -4063,6 +4063,9 @@
 Well done! fuel is a material that is burned to produce energy.
 Thanks for listening and learning with us today. We hope this episode helped you understand both the science and the English a little better. Keep practicing, stay curious, and remember that learning happens step by step.
 That’s the end of the video! I’m Bel — like and subscribe for Better English Learning!</t>
+  </si>
+  <si>
+    <t>https://youtu.be/XA1Fx0n4DRo</t>
   </si>
 </sst>
 </file>
@@ -5509,6 +5512,9 @@
       <c r="D73" t="s">
         <v>1089</v>
       </c>
+      <c r="E73" t="s">
+        <v>1100</v>
+      </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">

</xml_diff>